<commit_message>
Added API tests for Booking, DriverApp, LMFM, MM, Network, Notification, Scanning modules and updated Onboarding scenarios
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Credential" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="URL's" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Username</t>
   </si>
@@ -24,10 +24,70 @@
     <t>Password</t>
   </si>
   <si>
-    <t>Kuchbhi@123</t>
-  </si>
-  <si>
-    <t>VIJAY</t>
+    <t>mis.admin.400021</t>
+  </si>
+  <si>
+    <t>NewSecure$Pssword123</t>
+  </si>
+  <si>
+    <t>web (FE)</t>
+  </si>
+  <si>
+    <t>iam</t>
+  </si>
+  <si>
+    <t>booking</t>
+  </si>
+  <si>
+    <t>lmfm</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>network</t>
+  </si>
+  <si>
+    <t>notification</t>
+  </si>
+  <si>
+    <t>driverapp (BFF)</t>
+  </si>
+  <si>
+    <t>scanning</t>
+  </si>
+  <si>
+    <t>http://10.10.130.123:30000</t>
+  </si>
+  <si>
+    <t>http://10.10.130.123:30081</t>
+  </si>
+  <si>
+    <t>http://10.10.130.123:30082</t>
+  </si>
+  <si>
+    <t>http://10.10.130.123:30083</t>
+  </si>
+  <si>
+    <t>http://10.10.130.123:30084</t>
+  </si>
+  <si>
+    <t>http://10.10.130.123:30085</t>
+  </si>
+  <si>
+    <t>http://10.10.130.123:30086</t>
+  </si>
+  <si>
+    <t>http://10.10.130.123:30087</t>
+  </si>
+  <si>
+    <t>http://10.10.130.123:30088</t>
+  </si>
+  <si>
+    <t>Franchise</t>
+  </si>
+  <si>
+    <t>https://apidev.omone.in</t>
   </si>
 </sst>
 </file>
@@ -372,13 +432,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="11" width="27.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -386,17 +448,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId1" display="Kuchbhi@123"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -404,9 +475,90 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col min="9" max="9" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId2"/>
+    <hyperlink ref="C2" r:id="rId3"/>
+    <hyperlink ref="D2" r:id="rId4"/>
+    <hyperlink ref="E2" r:id="rId5"/>
+    <hyperlink ref="F2" r:id="rId6"/>
+    <hyperlink ref="G2" r:id="rId7"/>
+    <hyperlink ref="H2" r:id="rId8"/>
+    <hyperlink ref="I2" r:id="rId9"/>
+    <hyperlink ref="J2" r:id="rId10"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>